<commit_message>
Fix formulas inserted after shared ranges
</commit_message>
<xml_diff>
--- a/tests/fixtures/pm-report-shared-formulas-sanitized.xlsx
+++ b/tests/fixtures/pm-report-shared-formulas-sanitized.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="58" uniqueCount="40">
   <si>
     <t>SANITIZED SHARED-FORMULA PM TRACKER</t>
   </si>
@@ -69,7 +69,16 @@
     <t>Absolute helper</t>
   </si>
   <si>
+    <t>Sanitized filters</t>
+  </si>
+  <si>
+    <t>Sanitized guards</t>
+  </si>
+  <si>
     <t>Sanitized lubrication</t>
+  </si>
+  <si>
+    <t>Sanitized electrical</t>
   </si>
   <si>
     <t>Sanitized inspection</t>
@@ -245,8 +254,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" name="SanitizedPress23" displayName="SanitizedPress23" ref="A109:G112" totalsRowShown="1" headerRowCount="1">
-  <autoFilter ref="A109:G112">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" name="SanitizedPress23" displayName="SanitizedPress23" ref="A106:G112" totalsRowShown="1" headerRowCount="1">
+  <autoFilter ref="A106:G112">
     <filterColumn colId="0" hiddenButton="1"/>
     <filterColumn colId="1" hiddenButton="1"/>
     <filterColumn colId="2" hiddenButton="1"/>
@@ -704,44 +713,131 @@
         <v>13</v>
       </c>
     </row>
-    <row r="108" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A108" s="5" t="s">
+    <row r="105" spans="1:4" s="5" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A105" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B108" s="5" t="s">
+      <c r="B105" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C108" s="5" t="s">
+      <c r="C105" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="D108" s="5" t="s">
+      <c r="D105" s="5" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="109" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A109" s="2" t="s">
+    <row r="106" spans="1:8" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A106" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B109" s="2" t="s">
+      <c r="B106" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C109" s="2" t="s">
+      <c r="C106" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D109" s="2" t="s">
+      <c r="D106" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="E109" s="2" t="s">
+      <c r="E106" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="F109" s="2" t="s">
+      <c r="F106" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="G109" s="2" t="s">
+      <c r="G106" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="H109" s="2" t="s">
+      <c r="H106" s="2" t="s">
         <v>16</v>
+      </c>
+    </row>
+    <row r="107" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A107" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B107" s="3">
+        <v>75</v>
+      </c>
+      <c r="C107" s="3">
+        <v>0</v>
+      </c>
+      <c r="D107" s="3">
+        <v>5</v>
+      </c>
+      <c r="E107" s="4">
+        <f t="shared" ref="E107:E112" si="0">IF(OR(B107="",C107="",D107=""),"",B107-(D107-C107))</f>
+        <v>70</v>
+      </c>
+      <c r="F107" s="3" t="str">
+        <f t="shared" ref="F107:F112" si="1">IF(E107="","Needs Date",IF(E107&lt;0,"Past Due",IF(E107=0,"Due Today",IF(E107&lt;=7,"Due Soon","OK"))))</f>
+        <v>OK</v>
+      </c>
+      <c r="G107" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="H107">
+        <f>IF("B107"="B107",SUM(B102:B107)+'Reference Only'!$B$3,0)+$D107+E$6</f>
+        <v>75</v>
+      </c>
+    </row>
+    <row r="108" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A108" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B108" s="3">
+        <v>90</v>
+      </c>
+      <c r="C108" s="3">
+        <v>0</v>
+      </c>
+      <c r="D108" s="3">
+        <v>6</v>
+      </c>
+      <c r="E108" s="4">
+        <f t="shared" si="0"/>
+        <v>84</v>
+      </c>
+      <c r="F108" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>OK</v>
+      </c>
+      <c r="G108" s="3" t="s">
+        <v>18</v>
+      </c>
+      <c r="H108">
+        <f>IF("B108"="B108",SUM(B103:B108)+'Reference Only'!$B$3,0)+$D108+E$6</f>
+        <v>90</v>
+      </c>
+    </row>
+    <row r="109" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A109" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="B109" s="3">
+        <v>100</v>
+      </c>
+      <c r="C109" s="3">
+        <v>0</v>
+      </c>
+      <c r="D109" s="3">
+        <v>10</v>
+      </c>
+      <c r="E109" s="4">
+        <f t="shared" si="0"/>
+        <v>90</v>
+      </c>
+      <c r="F109" s="3" t="str">
+        <f t="shared" si="1"/>
+        <v>OK</v>
+      </c>
+      <c r="G109" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="H109">
+        <f>IF("B109"="B109",SUM(B104:B109)+'Reference Only'!$B$3,0)+$D109+E$6</f>
+        <v>100</v>
       </c>
     </row>
     <row r="110" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -749,28 +845,28 @@
         <v>12</v>
       </c>
       <c r="B110" s="3">
-        <v>100</v>
+        <v>125</v>
       </c>
       <c r="C110" s="3">
         <v>0</v>
       </c>
       <c r="D110" s="3">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E110" s="4">
-        <f t="shared" ref="E110:E112" si="0">IF(OR(B110="",C110="",D110=""),"",B110-(D110-C110))</f>
-        <v>90</v>
+        <f t="shared" si="0"/>
+        <v>110</v>
       </c>
       <c r="F110" s="3" t="str">
-        <f t="shared" ref="F110:F112" si="1">IF(E110="","Needs Date",IF(E110&lt;0,"Past Due",IF(E110=0,"Due Today",IF(E110&lt;=7,"Due Soon","OK"))))</f>
+        <f t="shared" si="1"/>
         <v>OK</v>
       </c>
       <c r="G110" s="3" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="H110">
-        <f>B110+$C$6+$D110+E$6</f>
-        <v>100</v>
+        <f>IF("B110"="B110",SUM(B105:B110)+'Reference Only'!$B$3,0)+$D110+E$6</f>
+        <v>125</v>
       </c>
     </row>
     <row r="111" ht="22" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
@@ -795,10 +891,10 @@
         <v>OK</v>
       </c>
       <c r="G111" s="3" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="H111">
-        <f>B111+$C$6+$D111+E$6</f>
+        <f>IF("B111"="B111",SUM(B106:B111)+'Reference Only'!$B$3,0)+$D111+E$6</f>
         <v>150</v>
       </c>
     </row>
@@ -824,10 +920,10 @@
         <v>OK</v>
       </c>
       <c r="G112" s="3" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="H112">
-        <f>B112+$C$6+$D112+E$6</f>
+        <f>IF("B112"="B112",SUM(B107:B112)+'Reference Only'!$B$3,0)+$D112+E$6</f>
         <v>200</v>
       </c>
     </row>
@@ -835,13 +931,13 @@
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
   </mergeCells>
-  <conditionalFormatting sqref="F110:F112">
+  <conditionalFormatting sqref="F107:F112">
     <cfRule type="expression" dxfId="0" priority="1">
-      <formula>F110="Past Due"</formula>
+      <formula>F107="Past Due"</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="2">
-    <dataValidation type="list" sqref="F110:F112">
+    <dataValidation type="list" sqref="F107:F112">
       <formula1>"Needs Date,Past Due,Due Today,Due Soon,OK"</formula1>
     </dataValidation>
     <dataValidation type="list" sqref="F6">
@@ -863,45 +959,45 @@
   <sheetData>
     <row r="2" spans="1:10" s="2" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="G2" s="2" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="H2" s="2" t="s">
         <v>5</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>29</v>
+        <v>32</v>
       </c>
       <c r="B3" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="C3" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="D3" s="6">
         <v>46204.5</v>
@@ -910,19 +1006,19 @@
         <v>46204.5</v>
       </c>
       <c r="F3" t="s">
-        <v>32</v>
+        <v>35</v>
       </c>
       <c r="G3" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="H3" t="s">
         <v>12</v>
       </c>
       <c r="I3" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="J3" t="s">
-        <v>34</v>
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -944,12 +1040,12 @@
   <sheetData>
     <row r="1" spans="1:1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
-        <v>35</v>
+        <v>38</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B3">
         <f>1+1</f>

</xml_diff>